<commit_message>
CASE_ZBT: rebuild 36 rows (01/07→05/08) từ export Jul+Aug + fapi 30d
Sửa lỗi ban đầu chỉ có 14 rows: export July CSV bị bỏ sót, fapi LSR/OI/klines
đủ 30 ngày. data_bad=1 còn 3 ngày (24-26/07). Phát hiện flush event 14-16/07:
vol 168M, f_avg âm, OI spike 11.2M.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_ZBT.xlsx
+++ b/docs/case_files/CASE_ZBT.xlsx
@@ -48,14 +48,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00BF8F00"/>
+        <bgColor rgb="00BF8F00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BF8F00"/>
-        <bgColor rgb="00BF8F00"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,8 +74,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -490,7 +490,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/08/2026 — cold-refresh lan dau tu 23/07</t>
+          <t>06/08/2026 — cold-refresh lan dau, window 07/07→05/08</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ZBTUSDT cold-refresh 23/07→05/08. Alpha DELISTED (ALPHA_435 fullyDelisted, HTTP 400). Export gap 24-26/07 (LSR/funding MISSING). Pin streak 10d (27/07→05/08), f_avg=5e-05 toan window. pos_r&gt;=3.0 tu 01/08 (5 ngay lien tuc, max 3.4081 ngay 02/08). div_avg3 4.1-4.2 tu 02/08. gLSR slope_5d &gt;1.0 toan window. OI floor 14d YES (05/08=min), 30d NO (06/08 tang len 10.1M). Depth ±2% snapshot 06/08T06:56 UTC: bid=$11,723 ask=$17,857 (~$29K). Nansen LOCKED. Unlock UNVERIFIED. Xem: docs/reports/_collect_zbt_20260806.md</t>
+          <t>ZBTUSDT cold-refresh 30d (07/07→05/08). Export: Jul+Aug CSV. LSR+OI: fapi 30d. Alpha DELISTED (ALPHA_435 fullyDelisted, HTTP 400). 07-16/07: fn tu export, LSR tu fapi. Pin streak 10d (27/07→05/08), f_avg=5e-05 tu 17/07. pos_r&gt;=3.0 tu 01/08 (5 ngay). div_avg3 4.1-4.2 tu 02/08. glsr_slope_5d &gt;1.0 toan window. Vol spike: 13/07=21M, 14/07=84M (flush event). OI spike 14/07: 11.2M (max 30d). Xem: docs/reports/_collect_zbt_20260806.md</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>O vang = operator dien/quyet · Header nau vang (sheet DAILY) = cot manual · Dong to cam (DAILY) = data_bad=1, so mang sai so (24-26/07: LSR/funding MISSING) · Cot cong thuc (ret_1d, div, slope, oi_vs_med14, oi_cycle_pos) da tinh san trong file nay.</t>
+          <t>O vang = operator dien/quyet · Header nau vang (DAILY) = cot manual · Dong to cam (DAILY) = data_bad=1 · Cot cong thuc da tinh san (ret_1d, div, slope, oi_vs_med14, oi_cycle_pos).</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO16"/>
+  <dimension ref="A1:AO38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -857,17 +857,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.108405</v>
+        <v>0.1409426362991903</v>
       </c>
       <c r="D3" t="n">
-        <v>22092107</v>
+        <v>215615573.95622</v>
       </c>
       <c r="E3" t="n">
-        <v>50.6</v>
+        <v>50.82509173013581</v>
       </c>
       <c r="F3" t="n">
         <v>5e-05</v>
@@ -885,25 +885,19 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>8725833</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1.0588</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.2896</v>
+        <v>8970308.81260642</v>
       </c>
       <c r="O3" t="n">
-        <v>2.3707</v>
+        <v>3.9917</v>
       </c>
       <c r="P3" t="n">
-        <v>0.578</v>
+        <v>0.8285</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.3951</v>
+        <v>0.6359</v>
       </c>
       <c r="R3" t="n">
-        <v>4.1016</v>
+        <v>4.818</v>
       </c>
       <c r="Z3" t="n">
         <v>0</v>
@@ -913,9 +907,6 @@
           <t>binance_spot</t>
         </is>
       </c>
-      <c r="AB3" t="n">
-        <v>2362962</v>
-      </c>
       <c r="AJ3" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -923,220 +914,220 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n">
-        <v>10524962</v>
-      </c>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n">
-        <v>9318649</v>
-      </c>
-      <c r="M4" s="3" t="n">
-        <v>1.1169</v>
-      </c>
-      <c r="N4" s="3" t="n">
-        <v>0.4584</v>
-      </c>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3" t="n"/>
-      <c r="T4" s="3" t="n"/>
-      <c r="U4" s="3" t="n"/>
-      <c r="V4" s="3" t="n"/>
-      <c r="W4" s="3" t="n"/>
-      <c r="X4" s="3" t="n"/>
-      <c r="Y4" s="3" t="n"/>
-      <c r="Z4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.1411777168101584</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.1668</v>
+      </c>
+      <c r="D4" t="n">
+        <v>73074368.9102</v>
+      </c>
+      <c r="E4" t="n">
+        <v>49.0578033993731</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="n">
+        <v>12560076.30049695</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2.6268</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.8918</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.8386</v>
+      </c>
+      <c r="R4" t="n">
+        <v>2.9455</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="inlineStr">
         <is>
           <t>binance_spot</t>
         </is>
       </c>
-      <c r="AB4" s="3" t="n">
-        <v>2037632</v>
-      </c>
-      <c r="AC4" s="3" t="n"/>
-      <c r="AD4" s="3" t="n"/>
-      <c r="AE4" s="3" t="n"/>
-      <c r="AF4" s="3" t="n"/>
-      <c r="AG4" s="3" t="n"/>
-      <c r="AH4" s="3" t="n"/>
-      <c r="AI4" s="3" t="n"/>
-      <c r="AJ4" s="3" t="inlineStr">
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>DELISTED</t>
         </is>
       </c>
-      <c r="AK4" s="3" t="n"/>
-      <c r="AL4" s="3" t="n"/>
-      <c r="AM4" s="3" t="n"/>
-      <c r="AN4" s="3" t="n"/>
-      <c r="AO4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n">
-        <v>4582927</v>
-      </c>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n">
-        <v>8545317</v>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>1.0242</v>
-      </c>
-      <c r="N5" s="3" t="n">
-        <v>0.2383</v>
-      </c>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n"/>
-      <c r="Q5" s="3" t="n"/>
-      <c r="R5" s="3" t="n"/>
-      <c r="S5" s="3" t="n"/>
-      <c r="T5" s="3" t="n"/>
-      <c r="U5" s="3" t="n"/>
-      <c r="V5" s="3" t="n"/>
-      <c r="W5" s="3" t="n"/>
-      <c r="X5" s="3" t="n"/>
-      <c r="Y5" s="3" t="n"/>
-      <c r="Z5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.137606567066772</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-2.5295</v>
+      </c>
+      <c r="D5" t="n">
+        <v>28342036.68354</v>
+      </c>
+      <c r="E5" t="n">
+        <v>48.40883272094256</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I5" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>10213390.28279734</v>
+      </c>
+      <c r="O5" t="n">
+        <v>3.0981</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.9673</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.8748</v>
+      </c>
+      <c r="R5" t="n">
+        <v>3.2028</v>
+      </c>
+      <c r="S5" t="n">
+        <v>3.6153</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="inlineStr">
         <is>
           <t>binance_spot</t>
         </is>
       </c>
-      <c r="AB5" s="3" t="n">
-        <v>1103203</v>
-      </c>
-      <c r="AC5" s="3" t="n"/>
-      <c r="AD5" s="3" t="n"/>
-      <c r="AE5" s="3" t="n"/>
-      <c r="AF5" s="3" t="n"/>
-      <c r="AG5" s="3" t="n"/>
-      <c r="AH5" s="3" t="n"/>
-      <c r="AI5" s="3" t="n"/>
-      <c r="AJ5" s="3" t="inlineStr">
+      <c r="AJ5" t="inlineStr">
         <is>
           <t>DELISTED</t>
         </is>
       </c>
-      <c r="AK5" s="3" t="n"/>
-      <c r="AL5" s="3" t="n"/>
-      <c r="AM5" s="3" t="n"/>
-      <c r="AN5" s="3" t="n"/>
-      <c r="AO5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n">
-        <v>9322656</v>
-      </c>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n">
-        <v>8452299</v>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>1.0009</v>
-      </c>
-      <c r="N6" s="3" t="n">
-        <v>0.2118</v>
-      </c>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="3" t="n"/>
-      <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3" t="n"/>
-      <c r="T6" s="3" t="n"/>
-      <c r="U6" s="3" t="n"/>
-      <c r="V6" s="3" t="n"/>
-      <c r="W6" s="3" t="n"/>
-      <c r="X6" s="3" t="n"/>
-      <c r="Y6" s="3" t="n"/>
-      <c r="Z6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.1391621868996169</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.1305</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16221897.6029</v>
+      </c>
+      <c r="E6" t="n">
+        <v>48.581446452799</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" t="n">
+        <v>10084405.98885297</v>
+      </c>
+      <c r="O6" t="n">
+        <v>3.567</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.9004</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.7486</v>
+      </c>
+      <c r="R6" t="n">
+        <v>3.9616</v>
+      </c>
+      <c r="S6" t="n">
+        <v>3.3672</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-0.4247</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.07190000000000001</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="inlineStr">
         <is>
           <t>binance_spot</t>
         </is>
       </c>
-      <c r="AB6" s="3" t="n">
-        <v>2345884</v>
-      </c>
-      <c r="AC6" s="3" t="n"/>
-      <c r="AD6" s="3" t="n"/>
-      <c r="AE6" s="3" t="n"/>
-      <c r="AF6" s="3" t="n"/>
-      <c r="AG6" s="3" t="n"/>
-      <c r="AH6" s="3" t="n"/>
-      <c r="AI6" s="3" t="n"/>
-      <c r="AJ6" s="3" t="inlineStr">
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>DELISTED</t>
         </is>
       </c>
-      <c r="AK6" s="3" t="n"/>
-      <c r="AL6" s="3" t="n"/>
-      <c r="AM6" s="3" t="n"/>
-      <c r="AN6" s="3" t="n"/>
-      <c r="AO6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.114577</v>
+        <v>0.1341215756660567</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-3.6221</v>
       </c>
       <c r="D7" t="n">
-        <v>6418842</v>
+        <v>12231550.25086</v>
       </c>
       <c r="E7" t="n">
-        <v>47.1</v>
+        <v>49.8202751697222</v>
       </c>
       <c r="F7" t="n">
         <v>5e-05</v>
@@ -1151,28 +1142,31 @@
         <v>6</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L7" t="n">
-        <v>8786963</v>
-      </c>
-      <c r="M7" t="n">
-        <v>1.0365</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.307</v>
+        <v>9443804.92664</v>
       </c>
       <c r="O7" t="n">
-        <v>2.754</v>
+        <v>3.7563</v>
       </c>
       <c r="P7" t="n">
-        <v>0.6614</v>
+        <v>0.8997000000000001</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.4482</v>
+        <v>0.6835</v>
       </c>
       <c r="R7" t="n">
-        <v>4.1639</v>
+        <v>4.1751</v>
+      </c>
+      <c r="S7" t="n">
+        <v>3.7658</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1.1295</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.007900000000000001</v>
       </c>
       <c r="Z7" t="n">
         <v>0</v>
@@ -1182,9 +1176,6 @@
           <t>binance_spot</t>
         </is>
       </c>
-      <c r="AB7" t="n">
-        <v>1483029</v>
-      </c>
       <c r="AJ7" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1194,20 +1185,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.112762</v>
+        <v>0.1294994761873012</v>
       </c>
       <c r="C8" t="n">
-        <v>-1.5841</v>
+        <v>-3.4462</v>
       </c>
       <c r="D8" t="n">
-        <v>4704342</v>
+        <v>8266242.16186</v>
       </c>
       <c r="E8" t="n">
-        <v>49</v>
+        <v>47.04966701672572</v>
       </c>
       <c r="F8" t="n">
         <v>5e-05</v>
@@ -1222,31 +1213,34 @@
         <v>6</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L8" t="n">
-        <v>8860722</v>
-      </c>
-      <c r="M8" t="n">
-        <v>1.0452</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.7156</v>
+        <v>9253510.60032</v>
       </c>
       <c r="O8" t="n">
-        <v>2.7491</v>
+        <v>3.9055</v>
       </c>
       <c r="P8" t="n">
-        <v>0.7097</v>
+        <v>0.8467</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.4575</v>
+        <v>0.6236</v>
       </c>
       <c r="R8" t="n">
-        <v>3.8736</v>
+        <v>4.6126</v>
+      </c>
+      <c r="S8" t="n">
+        <v>4.2424</v>
       </c>
       <c r="T8" t="n">
-        <v>1.1579</v>
+        <v>0.9807</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.8074</v>
+      </c>
+      <c r="V8" t="n">
+        <v>-0.1206</v>
       </c>
       <c r="Z8" t="n">
         <v>0</v>
@@ -1257,7 +1251,7 @@
         </is>
       </c>
       <c r="AB8" t="n">
-        <v>1323597</v>
+        <v>716534.88316</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
@@ -1268,20 +1262,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.112684</v>
+        <v>0.1250970910323144</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.0692</v>
+        <v>-3.3995</v>
       </c>
       <c r="D9" t="n">
-        <v>4983027</v>
+        <v>8115732.32616</v>
       </c>
       <c r="E9" t="n">
-        <v>47.1</v>
+        <v>46.34040952744668</v>
       </c>
       <c r="F9" t="n">
         <v>5e-05</v>
@@ -1296,31 +1290,34 @@
         <v>6</v>
       </c>
       <c r="K9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L9" t="n">
-        <v>8609763</v>
-      </c>
-      <c r="M9" t="n">
-        <v>1.0101</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.5598</v>
+        <v>8884858.756519999</v>
       </c>
       <c r="O9" t="n">
-        <v>2.6781</v>
+        <v>3.9472</v>
       </c>
       <c r="P9" t="n">
-        <v>0.7024</v>
+        <v>0.8389</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.4626</v>
+        <v>0.586</v>
       </c>
       <c r="R9" t="n">
-        <v>3.8128</v>
+        <v>4.7052</v>
       </c>
       <c r="S9" t="n">
-        <v>3.9456</v>
+        <v>4.4904</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.6988</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.3802</v>
+      </c>
+      <c r="V9" t="n">
+        <v>-0.0615</v>
       </c>
       <c r="Z9" t="n">
         <v>0</v>
@@ -1331,7 +1328,7 @@
         </is>
       </c>
       <c r="AB9" t="n">
-        <v>1541066</v>
+        <v>829159.4432</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
@@ -1342,20 +1339,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.116593</v>
+        <v>0.1230823693482214</v>
       </c>
       <c r="C10" t="n">
-        <v>3.469</v>
+        <v>-1.6105</v>
       </c>
       <c r="D10" t="n">
-        <v>6910711</v>
+        <v>11805105.99486</v>
       </c>
       <c r="E10" t="n">
-        <v>51.7</v>
+        <v>50.39954434901507</v>
       </c>
       <c r="F10" t="n">
         <v>5e-05</v>
@@ -1370,37 +1367,34 @@
         <v>6</v>
       </c>
       <c r="K10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L10" t="n">
-        <v>8476904</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.9945000000000001</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.4773</v>
+        <v>8447113.179749999</v>
       </c>
       <c r="O10" t="n">
-        <v>2.7421</v>
+        <v>4.0987</v>
       </c>
       <c r="P10" t="n">
-        <v>0.7077</v>
+        <v>0.7593</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.4535</v>
+        <v>0.5211</v>
       </c>
       <c r="R10" t="n">
-        <v>3.8747</v>
+        <v>5.398</v>
       </c>
       <c r="S10" t="n">
-        <v>3.8538</v>
+        <v>4.8883</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.5957</v>
       </c>
       <c r="U10" t="n">
-        <v>-0.0119</v>
+        <v>0.3424</v>
       </c>
       <c r="V10" t="n">
-        <v>0.0463</v>
+        <v>-0.1404</v>
       </c>
       <c r="Z10" t="n">
         <v>0</v>
@@ -1411,7 +1405,7 @@
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>2118287</v>
+        <v>1594423.90222</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
@@ -1422,20 +1416,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.11598</v>
+        <v>0.1208473023362933</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.5258</v>
+        <v>-1.8159</v>
       </c>
       <c r="D11" t="n">
-        <v>4394032</v>
+        <v>5336424.72396</v>
       </c>
       <c r="E11" t="n">
-        <v>48.6</v>
+        <v>46.80750960009656</v>
       </c>
       <c r="F11" t="n">
         <v>5e-05</v>
@@ -1450,37 +1444,34 @@
         <v>6</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L11" t="n">
-        <v>9143286</v>
-      </c>
-      <c r="M11" t="n">
-        <v>1.066</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.8911</v>
+        <v>8233642.01549</v>
       </c>
       <c r="O11" t="n">
-        <v>2.9249</v>
+        <v>4.0716</v>
       </c>
       <c r="P11" t="n">
-        <v>0.7106</v>
+        <v>0.8018</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.4643</v>
+        <v>0.5755</v>
       </c>
       <c r="R11" t="n">
-        <v>4.1161</v>
+        <v>5.0781</v>
       </c>
       <c r="S11" t="n">
-        <v>3.9351</v>
+        <v>5.049</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.7688</v>
       </c>
       <c r="U11" t="n">
-        <v>0.1758</v>
+        <v>0.1661</v>
       </c>
       <c r="V11" t="n">
-        <v>0.0009</v>
+        <v>-0.0449</v>
       </c>
       <c r="Z11" t="n">
         <v>0</v>
@@ -1491,7 +1482,7 @@
         </is>
       </c>
       <c r="AB11" t="n">
-        <v>1013687</v>
+        <v>789972.90392</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
@@ -1502,20 +1493,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.116464</v>
+        <v>0.1301326358147564</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4173</v>
+        <v>7.6835</v>
       </c>
       <c r="D12" t="n">
-        <v>2541983</v>
+        <v>14899276.9134</v>
       </c>
       <c r="E12" t="n">
-        <v>45.8</v>
+        <v>51.23519947069306</v>
       </c>
       <c r="F12" t="n">
         <v>5e-05</v>
@@ -1530,40 +1521,34 @@
         <v>6</v>
       </c>
       <c r="K12" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L12" t="n">
-        <v>8981809</v>
-      </c>
-      <c r="M12" t="n">
-        <v>1.0362</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0.7609</v>
+        <v>8232407.16918777</v>
       </c>
       <c r="O12" t="n">
-        <v>3.0691</v>
+        <v>4.2401</v>
       </c>
       <c r="P12" t="n">
-        <v>0.7699</v>
+        <v>0.7879</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.514</v>
+        <v>0.5564</v>
       </c>
       <c r="R12" t="n">
-        <v>3.9864</v>
+        <v>5.3815</v>
       </c>
       <c r="S12" t="n">
-        <v>3.9924</v>
+        <v>5.2833</v>
       </c>
       <c r="T12" t="n">
-        <v>1.1468</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="U12" t="n">
-        <v>0.391</v>
+        <v>0.2929</v>
       </c>
       <c r="V12" t="n">
-        <v>0.0675</v>
+        <v>-0.051</v>
       </c>
       <c r="Z12" t="n">
         <v>0</v>
@@ -1574,7 +1559,7 @@
         </is>
       </c>
       <c r="AB12" t="n">
-        <v>535087</v>
+        <v>2581808.51912</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
@@ -1585,20 +1570,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.122224</v>
+        <v>0.1254713414099807</v>
       </c>
       <c r="C13" t="n">
-        <v>4.9457</v>
+        <v>-3.582</v>
       </c>
       <c r="D13" t="n">
-        <v>6211662</v>
+        <v>9054733.7073</v>
       </c>
       <c r="E13" t="n">
-        <v>49.4</v>
+        <v>46.74575522988282</v>
       </c>
       <c r="F13" t="n">
         <v>5e-05</v>
@@ -1613,40 +1598,34 @@
         <v>6</v>
       </c>
       <c r="K13" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L13" t="n">
-        <v>8718627</v>
-      </c>
-      <c r="M13" t="n">
-        <v>1.0063</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.5741000000000001</v>
+        <v>8695521.688197</v>
       </c>
       <c r="O13" t="n">
-        <v>3.4081</v>
+        <v>4.0604</v>
       </c>
       <c r="P13" t="n">
-        <v>0.7544</v>
+        <v>0.8889</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.5117</v>
+        <v>0.6506999999999999</v>
       </c>
       <c r="R13" t="n">
-        <v>4.5176</v>
+        <v>4.5679</v>
       </c>
       <c r="S13" t="n">
-        <v>4.2069</v>
+        <v>4.9916</v>
       </c>
       <c r="T13" t="n">
-        <v>1.1185</v>
+        <v>1.0435</v>
       </c>
       <c r="U13" t="n">
-        <v>0.666</v>
+        <v>-0.0383</v>
       </c>
       <c r="V13" t="n">
-        <v>0.0467</v>
+        <v>0.1296</v>
       </c>
       <c r="Z13" t="n">
         <v>0</v>
@@ -1657,7 +1636,7 @@
         </is>
       </c>
       <c r="AB13" t="n">
-        <v>1688089</v>
+        <v>981579.05883</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
@@ -1668,20 +1647,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.118481</v>
+        <v>0.1176295917994711</v>
       </c>
       <c r="C14" t="n">
-        <v>-3.0624</v>
+        <v>-6.2498</v>
       </c>
       <c r="D14" t="n">
-        <v>3507809</v>
+        <v>6099510.03778</v>
       </c>
       <c r="E14" t="n">
-        <v>47.1</v>
+        <v>46.17733931511867</v>
       </c>
       <c r="F14" t="n">
         <v>5e-05</v>
@@ -1696,40 +1675,34 @@
         <v>6</v>
       </c>
       <c r="K14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="L14" t="n">
-        <v>9297648</v>
-      </c>
-      <c r="M14" t="n">
-        <v>1.066</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0.9851</v>
+        <v>8249896.11618</v>
       </c>
       <c r="O14" t="n">
-        <v>3.2607</v>
+        <v>3.9692</v>
       </c>
       <c r="P14" t="n">
-        <v>0.8245</v>
+        <v>0.8598</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.5586</v>
+        <v>0.6279</v>
       </c>
       <c r="R14" t="n">
-        <v>3.9548</v>
+        <v>4.6164</v>
       </c>
       <c r="S14" t="n">
-        <v>4.1459</v>
+        <v>4.8371</v>
       </c>
       <c r="T14" t="n">
-        <v>1.2075</v>
+        <v>1.0715</v>
       </c>
       <c r="U14" t="n">
-        <v>0.3358</v>
+        <v>-0.1024</v>
       </c>
       <c r="V14" t="n">
-        <v>0.1139</v>
+        <v>0.058</v>
       </c>
       <c r="Z14" t="n">
         <v>0</v>
@@ -1740,7 +1713,7 @@
         </is>
       </c>
       <c r="AB14" t="n">
-        <v>860103</v>
+        <v>762823.51981</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
@@ -1751,20 +1724,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.111582</v>
+        <v>0.1309449800837556</v>
       </c>
       <c r="C15" t="n">
-        <v>-5.8229</v>
+        <v>11.3198</v>
       </c>
       <c r="D15" t="n">
-        <v>3564479</v>
+        <v>42466521.88574</v>
       </c>
       <c r="E15" t="n">
-        <v>50</v>
+        <v>52.21305715091059</v>
       </c>
       <c r="F15" t="n">
         <v>5e-05</v>
@@ -1779,40 +1752,34 @@
         <v>6</v>
       </c>
       <c r="K15" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L15" t="n">
-        <v>8579454</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0.9836</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.1468</v>
+        <v>8028748.0625</v>
       </c>
       <c r="O15" t="n">
-        <v>3.3595</v>
+        <v>3.9621</v>
       </c>
       <c r="P15" t="n">
-        <v>0.8175</v>
+        <v>0.7409</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.5571</v>
+        <v>0.5161</v>
       </c>
       <c r="R15" t="n">
-        <v>4.1095</v>
+        <v>5.3477</v>
       </c>
       <c r="S15" t="n">
-        <v>4.1847</v>
+        <v>4.8167</v>
       </c>
       <c r="T15" t="n">
-        <v>1.2284</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="U15" t="n">
-        <v>0.2904</v>
+        <v>-0.278</v>
       </c>
       <c r="V15" t="n">
-        <v>0.0476</v>
+        <v>-0.047</v>
       </c>
       <c r="Z15" t="n">
         <v>0</v>
@@ -1823,7 +1790,7 @@
         </is>
       </c>
       <c r="AB15" t="n">
-        <v>957955</v>
+        <v>4503531.19663</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
@@ -1834,26 +1801,26 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.117641</v>
+        <v>0.1337539642687834</v>
       </c>
       <c r="C16" t="n">
-        <v>5.4301</v>
+        <v>2.1452</v>
       </c>
       <c r="D16" t="n">
-        <v>15060833</v>
+        <v>168164207.84728</v>
       </c>
       <c r="E16" t="n">
-        <v>50.6</v>
+        <v>49.37939415999092</v>
       </c>
       <c r="F16" t="n">
-        <v>5e-05</v>
+        <v>3.283166666666667e-05</v>
       </c>
       <c r="G16" t="n">
-        <v>5e-05</v>
+        <v>-3.005e-05</v>
       </c>
       <c r="H16" t="n">
         <v>5e-05</v>
@@ -1861,41 +1828,38 @@
       <c r="I16" t="n">
         <v>6</v>
       </c>
-      <c r="K16" t="n">
-        <v>10</v>
-      </c>
       <c r="L16" t="n">
-        <v>7889446</v>
+        <v>11221125.44926848</v>
       </c>
       <c r="M16" t="n">
-        <v>0.9045</v>
+        <v>1.2569</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>0.7045</v>
       </c>
       <c r="O16" t="n">
-        <v>3.4072</v>
+        <v>2.8336</v>
       </c>
       <c r="P16" t="n">
-        <v>0.7467</v>
+        <v>0.6731</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.4914</v>
+        <v>0.5708</v>
       </c>
       <c r="R16" t="n">
-        <v>4.563</v>
+        <v>4.2098</v>
       </c>
       <c r="S16" t="n">
-        <v>4.1978</v>
+        <v>4.7343</v>
       </c>
       <c r="T16" t="n">
-        <v>1.0584</v>
+        <v>0.9918</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.0009</v>
+        <v>-1.2268</v>
       </c>
       <c r="V16" t="n">
-        <v>-0.0077</v>
+        <v>-0.2158</v>
       </c>
       <c r="Z16" t="n">
         <v>0</v>
@@ -1906,9 +1870,1847 @@
         </is>
       </c>
       <c r="AB16" t="n">
-        <v>4776726</v>
+        <v>9717927.89711</v>
       </c>
       <c r="AJ16" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.09284590614145299</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-30.5846</v>
+      </c>
+      <c r="D17" t="n">
+        <v>133070146.1998</v>
+      </c>
+      <c r="E17" t="n">
+        <v>49.56457192034431</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-0.00040081</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-0.00067596</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-3.87e-05</v>
+      </c>
+      <c r="I17" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" t="n">
+        <v>8437412.341399999</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.9599</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.0902</v>
+      </c>
+      <c r="O17" t="n">
+        <v>3.0427</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.7334000000000001</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.517</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.1488</v>
+      </c>
+      <c r="S17" t="n">
+        <v>4.5815</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0.9292</v>
+      </c>
+      <c r="U17" t="n">
+        <v>-0.9265</v>
+      </c>
+      <c r="V17" t="n">
+        <v>-0.1264</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB17" t="n">
+        <v>13620381.48736</v>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.08991763877380129</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-3.1539</v>
+      </c>
+      <c r="D18" t="n">
+        <v>36649806.6148</v>
+      </c>
+      <c r="E18" t="n">
+        <v>48.71870880325287</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-0.000341675</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-0.00127902</v>
+      </c>
+      <c r="H18" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I18" t="n">
+        <v>6</v>
+      </c>
+      <c r="L18" t="n">
+        <v>7765104.16145</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.9059</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1.7856</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.6748</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.5337</v>
+      </c>
+      <c r="R18" t="n">
+        <v>2.6461</v>
+      </c>
+      <c r="S18" t="n">
+        <v>3.6813</v>
+      </c>
+      <c r="T18" t="n">
+        <v>0.8202</v>
+      </c>
+      <c r="U18" t="n">
+        <v>-2.1765</v>
+      </c>
+      <c r="V18" t="n">
+        <v>-0.06610000000000001</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB18" t="n">
+        <v>4483317.54093</v>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.0899405742615771</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="D19" t="n">
+        <v>21212000.01966</v>
+      </c>
+      <c r="E19" t="n">
+        <v>49.76644703601743</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I19" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" t="n">
+        <v>7747592.84777244</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.9177</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1.8171</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.6223</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.4665</v>
+      </c>
+      <c r="R19" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="S19" t="n">
+        <v>3.2728</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="U19" t="n">
+        <v>-1.0165</v>
+      </c>
+      <c r="V19" t="n">
+        <v>-0.0508</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB19" t="n">
+        <v>2979494.89578</v>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.0958041212387999</v>
+      </c>
+      <c r="C20" t="n">
+        <v>6.5194</v>
+      </c>
+      <c r="D20" t="n">
+        <v>66020582.01406</v>
+      </c>
+      <c r="E20" t="n">
+        <v>48.7543999517234</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4.187666666666666e-05</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1.26e-06</v>
+      </c>
+      <c r="H20" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I20" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" t="n">
+        <v>7708392.699</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.9239000000000001</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>1.8365</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.6075</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="R20" t="n">
+        <v>3.023</v>
+      </c>
+      <c r="S20" t="n">
+        <v>2.8558</v>
+      </c>
+      <c r="T20" t="n">
+        <v>0.8603</v>
+      </c>
+      <c r="U20" t="n">
+        <v>-1.2062</v>
+      </c>
+      <c r="V20" t="n">
+        <v>-0.1259</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB20" t="n">
+        <v>7559250.35841</v>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.1004155086699476</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4.8133</v>
+      </c>
+      <c r="D21" t="n">
+        <v>49651495.39478</v>
+      </c>
+      <c r="E21" t="n">
+        <v>48.21771527158048</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G21" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H21" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" t="n">
+        <v>9173494.616175471</v>
+      </c>
+      <c r="M21" t="n">
+        <v>1.0995</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.4171</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1.9546</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0.5903</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.4318</v>
+      </c>
+      <c r="R21" t="n">
+        <v>3.3112</v>
+      </c>
+      <c r="S21" t="n">
+        <v>3.0813</v>
+      </c>
+      <c r="T21" t="n">
+        <v>0.7565</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="V21" t="n">
+        <v>-0.08450000000000001</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB21" t="n">
+        <v>3816424.84366</v>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.09147927028306831</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-8.8993</v>
+      </c>
+      <c r="D22" t="n">
+        <v>21054968.01188</v>
+      </c>
+      <c r="E22" t="n">
+        <v>49.86771560453432</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G22" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H22" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I22" t="n">
+        <v>6</v>
+      </c>
+      <c r="K22" t="n">
+        <v>4</v>
+      </c>
+      <c r="L22" t="n">
+        <v>8087757.9106952</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.9813</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="O22" t="n">
+        <v>2.1008</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.6598000000000001</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.4445</v>
+      </c>
+      <c r="R22" t="n">
+        <v>3.184</v>
+      </c>
+      <c r="S22" t="n">
+        <v>3.1718</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0.8598</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0.2837</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB22" t="n">
+        <v>1667068.5947</v>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.09512081178750501</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3.9807</v>
+      </c>
+      <c r="D23" t="n">
+        <v>30287680.2147</v>
+      </c>
+      <c r="E23" t="n">
+        <v>48.69974426449438</v>
+      </c>
+      <c r="F23" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G23" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H23" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I23" t="n">
+        <v>6</v>
+      </c>
+      <c r="K23" t="n">
+        <v>5</v>
+      </c>
+      <c r="L23" t="n">
+        <v>7909721.98426</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.9607</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.0573</v>
+      </c>
+      <c r="O23" t="n">
+        <v>2.2997</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.6139</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.4088</v>
+      </c>
+      <c r="R23" t="n">
+        <v>3.746</v>
+      </c>
+      <c r="S23" t="n">
+        <v>3.4094</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0.4632</v>
+      </c>
+      <c r="V23" t="n">
+        <v>0.0064</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB23" t="n">
+        <v>2615428.9535</v>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.1015470670877675</v>
+      </c>
+      <c r="C24" t="n">
+        <v>6.7559</v>
+      </c>
+      <c r="D24" t="n">
+        <v>19437512.22416</v>
+      </c>
+      <c r="E24" t="n">
+        <v>51.52759916004675</v>
+      </c>
+      <c r="F24" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G24" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H24" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I24" t="n">
+        <v>6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>6</v>
+      </c>
+      <c r="L24" t="n">
+        <v>8502283.62662</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1.0327</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="O24" t="n">
+        <v>2.4132</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.5504</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.3829</v>
+      </c>
+      <c r="R24" t="n">
+        <v>4.3844</v>
+      </c>
+      <c r="S24" t="n">
+        <v>3.7354</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0.8208</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0.4586</v>
+      </c>
+      <c r="V24" t="n">
+        <v>-0.0399</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB24" t="n">
+        <v>1971541.38956</v>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.1084049731823625</v>
+      </c>
+      <c r="C25" t="n">
+        <v>6.7534</v>
+      </c>
+      <c r="D25" t="n">
+        <v>22092106.83824</v>
+      </c>
+      <c r="E25" t="n">
+        <v>50.5707367733576</v>
+      </c>
+      <c r="F25" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G25" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H25" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I25" t="n">
+        <v>6</v>
+      </c>
+      <c r="K25" t="n">
+        <v>7</v>
+      </c>
+      <c r="L25" t="n">
+        <v>8725832.601600001</v>
+      </c>
+      <c r="M25" t="n">
+        <v>1.0588</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.2896</v>
+      </c>
+      <c r="O25" t="n">
+        <v>2.3707</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.578</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.3951</v>
+      </c>
+      <c r="R25" t="n">
+        <v>4.1016</v>
+      </c>
+      <c r="S25" t="n">
+        <v>4.0657</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0.8899</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0.2699</v>
+      </c>
+      <c r="V25" t="n">
+        <v>-0.0818</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB25" t="n">
+        <v>2362962.39597</v>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>0.10923</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>0.7611</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>10524961.71948</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>48.3596</v>
+      </c>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n">
+        <v>9318648.8989894</v>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>1.1169</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>0.4584</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>2.5344</v>
+      </c>
+      <c r="P26" s="3" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="Q26" s="3" t="n">
+        <v>0.4013</v>
+      </c>
+      <c r="R26" s="3" t="n">
+        <v>4.5056</v>
+      </c>
+      <c r="S26" s="3" t="n">
+        <v>4.3281</v>
+      </c>
+      <c r="T26" s="3" t="n">
+        <v>0.9294</v>
+      </c>
+      <c r="U26" s="3" t="n">
+        <v>0.2347</v>
+      </c>
+      <c r="V26" s="3" t="n">
+        <v>-0.0514</v>
+      </c>
+      <c r="W26" s="3" t="n"/>
+      <c r="X26" s="3" t="n"/>
+      <c r="Y26" s="3" t="n"/>
+      <c r="Z26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA26" s="3" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB26" s="3" t="n">
+        <v>2037632.16795</v>
+      </c>
+      <c r="AC26" s="3" t="n"/>
+      <c r="AD26" s="3" t="n"/>
+      <c r="AE26" s="3" t="n"/>
+      <c r="AF26" s="3" t="n"/>
+      <c r="AG26" s="3" t="n"/>
+      <c r="AH26" s="3" t="n"/>
+      <c r="AI26" s="3" t="n"/>
+      <c r="AJ26" s="3" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+      <c r="AK26" s="3" t="n"/>
+      <c r="AL26" s="3" t="n"/>
+      <c r="AM26" s="3" t="n"/>
+      <c r="AN26" s="3" t="n"/>
+      <c r="AO26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>0.10857</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>-0.6042</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>4582926.60191</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>49.1967</v>
+      </c>
+      <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n">
+        <v>8545316.532059999</v>
+      </c>
+      <c r="M27" s="3" t="n">
+        <v>1.0242</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>0.2383</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>2.5636</v>
+      </c>
+      <c r="P27" s="3" t="n">
+        <v>0.6264999999999999</v>
+      </c>
+      <c r="Q27" s="3" t="n">
+        <v>0.4263</v>
+      </c>
+      <c r="R27" s="3" t="n">
+        <v>4.0919</v>
+      </c>
+      <c r="S27" s="3" t="n">
+        <v>4.2268</v>
+      </c>
+      <c r="T27" s="3" t="n">
+        <v>0.9591</v>
+      </c>
+      <c r="U27" s="3" t="n">
+        <v>0.1504</v>
+      </c>
+      <c r="V27" s="3" t="n">
+        <v>0.0761</v>
+      </c>
+      <c r="W27" s="3" t="n"/>
+      <c r="X27" s="3" t="n"/>
+      <c r="Y27" s="3" t="n"/>
+      <c r="Z27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA27" s="3" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB27" s="3" t="n">
+        <v>1103202.75839</v>
+      </c>
+      <c r="AC27" s="3" t="n"/>
+      <c r="AD27" s="3" t="n"/>
+      <c r="AE27" s="3" t="n"/>
+      <c r="AF27" s="3" t="n"/>
+      <c r="AG27" s="3" t="n"/>
+      <c r="AH27" s="3" t="n"/>
+      <c r="AI27" s="3" t="n"/>
+      <c r="AJ27" s="3" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+      <c r="AK27" s="3" t="n"/>
+      <c r="AL27" s="3" t="n"/>
+      <c r="AM27" s="3" t="n"/>
+      <c r="AN27" s="3" t="n"/>
+      <c r="AO27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>0.11335</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>4.4027</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>9322656.45967</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>51.0288</v>
+      </c>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n">
+        <v>8452298.983911119</v>
+      </c>
+      <c r="M28" s="3" t="n">
+        <v>1.0009</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>0.2118</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>2.6128</v>
+      </c>
+      <c r="P28" s="3" t="n">
+        <v>0.6491</v>
+      </c>
+      <c r="Q28" s="3" t="n">
+        <v>0.4323</v>
+      </c>
+      <c r="R28" s="3" t="n">
+        <v>4.0253</v>
+      </c>
+      <c r="S28" s="3" t="n">
+        <v>4.195</v>
+      </c>
+      <c r="T28" s="3" t="n">
+        <v>1.0575</v>
+      </c>
+      <c r="U28" s="3" t="n">
+        <v>0.2421</v>
+      </c>
+      <c r="V28" s="3" t="n">
+        <v>0.0711</v>
+      </c>
+      <c r="W28" s="3" t="n"/>
+      <c r="X28" s="3" t="n"/>
+      <c r="Y28" s="3" t="n"/>
+      <c r="Z28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA28" s="3" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB28" s="3" t="n">
+        <v>2345884.3215</v>
+      </c>
+      <c r="AC28" s="3" t="n"/>
+      <c r="AD28" s="3" t="n"/>
+      <c r="AE28" s="3" t="n"/>
+      <c r="AF28" s="3" t="n"/>
+      <c r="AG28" s="3" t="n"/>
+      <c r="AH28" s="3" t="n"/>
+      <c r="AI28" s="3" t="n"/>
+      <c r="AJ28" s="3" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+      <c r="AK28" s="3" t="n"/>
+      <c r="AL28" s="3" t="n"/>
+      <c r="AM28" s="3" t="n"/>
+      <c r="AN28" s="3" t="n"/>
+      <c r="AO28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.1145771354349844</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1.0826</v>
+      </c>
+      <c r="D29" t="n">
+        <v>6418842.22915</v>
+      </c>
+      <c r="E29" t="n">
+        <v>47.05072540506195</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G29" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H29" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I29" t="n">
+        <v>6</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" t="n">
+        <v>8786963.355901901</v>
+      </c>
+      <c r="M29" t="n">
+        <v>1.0365</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0.307</v>
+      </c>
+      <c r="O29" t="n">
+        <v>2.754</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0.6614</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0.4482</v>
+      </c>
+      <c r="R29" t="n">
+        <v>4.1639</v>
+      </c>
+      <c r="S29" t="n">
+        <v>4.0942</v>
+      </c>
+      <c r="T29" t="n">
+        <v>1.1705</v>
+      </c>
+      <c r="U29" t="n">
+        <v>0.2196</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0.0989</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB29" t="n">
+        <v>1483028.91662</v>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.1127621379125496</v>
+      </c>
+      <c r="C30" t="n">
+        <v>-1.5841</v>
+      </c>
+      <c r="D30" t="n">
+        <v>4704341.89904</v>
+      </c>
+      <c r="E30" t="n">
+        <v>49.04198940073379</v>
+      </c>
+      <c r="F30" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G30" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H30" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I30" t="n">
+        <v>6</v>
+      </c>
+      <c r="K30" t="n">
+        <v>2</v>
+      </c>
+      <c r="L30" t="n">
+        <v>8860722.138853321</v>
+      </c>
+      <c r="M30" t="n">
+        <v>1.0452</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.7156</v>
+      </c>
+      <c r="O30" t="n">
+        <v>2.7491</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0.7097</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0.4575</v>
+      </c>
+      <c r="R30" t="n">
+        <v>3.8736</v>
+      </c>
+      <c r="S30" t="n">
+        <v>4.0174</v>
+      </c>
+      <c r="T30" t="n">
+        <v>1.1579</v>
+      </c>
+      <c r="U30" t="n">
+        <v>0.1855</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0.0832</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB30" t="n">
+        <v>1323596.82829</v>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.1126842754135239</v>
+      </c>
+      <c r="C31" t="n">
+        <v>-0.06909999999999999</v>
+      </c>
+      <c r="D31" t="n">
+        <v>4983027.11886</v>
+      </c>
+      <c r="E31" t="n">
+        <v>47.11233340385022</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G31" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H31" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I31" t="n">
+        <v>6</v>
+      </c>
+      <c r="K31" t="n">
+        <v>3</v>
+      </c>
+      <c r="L31" t="n">
+        <v>8609762.918723291</v>
+      </c>
+      <c r="M31" t="n">
+        <v>1.0101</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0.5598</v>
+      </c>
+      <c r="O31" t="n">
+        <v>2.6781</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0.7024</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0.4626</v>
+      </c>
+      <c r="R31" t="n">
+        <v>3.8128</v>
+      </c>
+      <c r="S31" t="n">
+        <v>3.9456</v>
+      </c>
+      <c r="T31" t="n">
+        <v>1.1528</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0.0653</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0.0533</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB31" t="n">
+        <v>1541065.83729</v>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0.1165926131962741</v>
+      </c>
+      <c r="C32" t="n">
+        <v>3.4684</v>
+      </c>
+      <c r="D32" t="n">
+        <v>6910711.29782</v>
+      </c>
+      <c r="E32" t="n">
+        <v>51.69082125603865</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H32" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I32" t="n">
+        <v>6</v>
+      </c>
+      <c r="K32" t="n">
+        <v>4</v>
+      </c>
+      <c r="L32" t="n">
+        <v>8476904.2030157</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.9945000000000001</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.4773</v>
+      </c>
+      <c r="O32" t="n">
+        <v>2.7421</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0.7077</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.4535</v>
+      </c>
+      <c r="R32" t="n">
+        <v>3.8747</v>
+      </c>
+      <c r="S32" t="n">
+        <v>3.8538</v>
+      </c>
+      <c r="T32" t="n">
+        <v>1.0638</v>
+      </c>
+      <c r="U32" t="n">
+        <v>-0.0119</v>
+      </c>
+      <c r="V32" t="n">
+        <v>0.0463</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB32" t="n">
+        <v>2118286.95634</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0.1159795815646512</v>
+      </c>
+      <c r="C33" t="n">
+        <v>-0.5258</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4394032.465869999</v>
+      </c>
+      <c r="E33" t="n">
+        <v>48.56231675325343</v>
+      </c>
+      <c r="F33" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G33" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H33" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I33" t="n">
+        <v>6</v>
+      </c>
+      <c r="K33" t="n">
+        <v>5</v>
+      </c>
+      <c r="L33" t="n">
+        <v>9143285.61682374</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0.8911</v>
+      </c>
+      <c r="O33" t="n">
+        <v>2.9249</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0.7106</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.4643</v>
+      </c>
+      <c r="R33" t="n">
+        <v>4.1161</v>
+      </c>
+      <c r="S33" t="n">
+        <v>3.9351</v>
+      </c>
+      <c r="T33" t="n">
+        <v>1.074</v>
+      </c>
+      <c r="U33" t="n">
+        <v>0.1758</v>
+      </c>
+      <c r="V33" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB33" t="n">
+        <v>1013687.05613</v>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.1164637776196714</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.4175</v>
+      </c>
+      <c r="D34" t="n">
+        <v>2541982.89949</v>
+      </c>
+      <c r="E34" t="n">
+        <v>45.82588439243729</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G34" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H34" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I34" t="n">
+        <v>6</v>
+      </c>
+      <c r="K34" t="n">
+        <v>6</v>
+      </c>
+      <c r="L34" t="n">
+        <v>8981809.140009999</v>
+      </c>
+      <c r="M34" t="n">
+        <v>1.0362</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0.7609</v>
+      </c>
+      <c r="O34" t="n">
+        <v>3.0691</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0.7699</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="R34" t="n">
+        <v>3.9864</v>
+      </c>
+      <c r="S34" t="n">
+        <v>3.9924</v>
+      </c>
+      <c r="T34" t="n">
+        <v>1.1468</v>
+      </c>
+      <c r="U34" t="n">
+        <v>0.391</v>
+      </c>
+      <c r="V34" t="n">
+        <v>0.0675</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB34" t="n">
+        <v>535087.36674</v>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.1222236760030807</v>
+      </c>
+      <c r="C35" t="n">
+        <v>4.9457</v>
+      </c>
+      <c r="D35" t="n">
+        <v>6211661.68417</v>
+      </c>
+      <c r="E35" t="n">
+        <v>49.36452478606511</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G35" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H35" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I35" t="n">
+        <v>6</v>
+      </c>
+      <c r="K35" t="n">
+        <v>7</v>
+      </c>
+      <c r="L35" t="n">
+        <v>8718627.472411521</v>
+      </c>
+      <c r="M35" t="n">
+        <v>1.0063</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.5741000000000001</v>
+      </c>
+      <c r="O35" t="n">
+        <v>3.4081</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0.7544</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0.5117</v>
+      </c>
+      <c r="R35" t="n">
+        <v>4.5176</v>
+      </c>
+      <c r="S35" t="n">
+        <v>4.2069</v>
+      </c>
+      <c r="T35" t="n">
+        <v>1.1185</v>
+      </c>
+      <c r="U35" t="n">
+        <v>0.666</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB35" t="n">
+        <v>1688089.23149</v>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.1184813530492571</v>
+      </c>
+      <c r="C36" t="n">
+        <v>-3.0619</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3507809.17447</v>
+      </c>
+      <c r="E36" t="n">
+        <v>47.05913494626502</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G36" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H36" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I36" t="n">
+        <v>6</v>
+      </c>
+      <c r="K36" t="n">
+        <v>8</v>
+      </c>
+      <c r="L36" t="n">
+        <v>9297647.830800001</v>
+      </c>
+      <c r="M36" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0.9851</v>
+      </c>
+      <c r="O36" t="n">
+        <v>3.2607</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0.8245</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0.5586</v>
+      </c>
+      <c r="R36" t="n">
+        <v>3.9548</v>
+      </c>
+      <c r="S36" t="n">
+        <v>4.1459</v>
+      </c>
+      <c r="T36" t="n">
+        <v>1.2075</v>
+      </c>
+      <c r="U36" t="n">
+        <v>0.3358</v>
+      </c>
+      <c r="V36" t="n">
+        <v>0.1139</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
+        <v>860103.143</v>
+      </c>
+      <c r="AJ36" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.1115824715239967</v>
+      </c>
+      <c r="C37" t="n">
+        <v>-5.8228</v>
+      </c>
+      <c r="D37" t="n">
+        <v>3564478.84368</v>
+      </c>
+      <c r="E37" t="n">
+        <v>49.95245483209048</v>
+      </c>
+      <c r="F37" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G37" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H37" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I37" t="n">
+        <v>6</v>
+      </c>
+      <c r="K37" t="n">
+        <v>9</v>
+      </c>
+      <c r="L37" t="n">
+        <v>8579453.65236252</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.9836</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0.1468</v>
+      </c>
+      <c r="O37" t="n">
+        <v>3.3595</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0.5571</v>
+      </c>
+      <c r="R37" t="n">
+        <v>4.1095</v>
+      </c>
+      <c r="S37" t="n">
+        <v>4.1847</v>
+      </c>
+      <c r="T37" t="n">
+        <v>1.2284</v>
+      </c>
+      <c r="U37" t="n">
+        <v>0.2904</v>
+      </c>
+      <c r="V37" t="n">
+        <v>0.0476</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB37" t="n">
+        <v>957955.40446</v>
+      </c>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>DELISTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.1176408335547829</v>
+      </c>
+      <c r="C38" t="n">
+        <v>5.4295</v>
+      </c>
+      <c r="D38" t="n">
+        <v>15060833.48766</v>
+      </c>
+      <c r="E38" t="n">
+        <v>50.5831191935165</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="G38" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H38" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I38" t="n">
+        <v>6</v>
+      </c>
+      <c r="K38" t="n">
+        <v>10</v>
+      </c>
+      <c r="L38" t="n">
+        <v>7889445.69524712</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.9045</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>3.4072</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0.7467</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0.4914</v>
+      </c>
+      <c r="R38" t="n">
+        <v>4.563</v>
+      </c>
+      <c r="S38" t="n">
+        <v>4.1978</v>
+      </c>
+      <c r="T38" t="n">
+        <v>1.0584</v>
+      </c>
+      <c r="U38" t="n">
+        <v>-0.0009</v>
+      </c>
+      <c r="V38" t="n">
+        <v>-0.0077</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>binance_spot</t>
+        </is>
+      </c>
+      <c r="AB38" t="n">
+        <v>4776726.25304</v>
+      </c>
+      <c r="AJ38" t="inlineStr">
         <is>
           <t>DELISTED</t>
         </is>
@@ -2022,7 +3824,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>E. OUTCOME — dien tai moc; verdict_check: verdict luc mo DUNG/SAI o diem nao</t>
+          <t>E. OUTCOME — dien tai moc; verdict_check</t>
         </is>
       </c>
     </row>
@@ -2064,7 +3866,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>J. TOKENOMICS / UNLOCK — dong cung co lich, MM danh quanh no</t>
+          <t>J. TOKENOMICS / UNLOCK — dong cung co lich</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ZBT: patch taker_spot_pct 36 ngày (fix k[9]→k[10])
Root cause: probe cũ dùng k[9] (base tokens) ÷ k[7] (USDT) → đơn vị lệch → ~400%.
Fix: k[10] (takerBuyQuoteAssetVolume, USDT) ÷ k[7] (quoteVol, USDT) → 42–55% hợp lệ.
Đồng bộ logic với spot_collector.py (đã duyệt 21/07).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_ZBT.xlsx
+++ b/docs/case_files/CASE_ZBT.xlsx
@@ -907,6 +907,9 @@
           <t>binance_spot</t>
         </is>
       </c>
+      <c r="AC3" t="n">
+        <v>49.14</v>
+      </c>
       <c r="AJ3" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -969,6 +972,9 @@
           <t>binance_spot</t>
         </is>
       </c>
+      <c r="AC4" t="n">
+        <v>46.45</v>
+      </c>
       <c r="AJ4" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1034,6 +1040,9 @@
           <t>binance_spot</t>
         </is>
       </c>
+      <c r="AC5" t="n">
+        <v>45.55</v>
+      </c>
       <c r="AJ5" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1105,6 +1114,9 @@
           <t>binance_spot</t>
         </is>
       </c>
+      <c r="AC6" t="n">
+        <v>46.71</v>
+      </c>
       <c r="AJ6" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1176,6 +1188,9 @@
           <t>binance_spot</t>
         </is>
       </c>
+      <c r="AC7" t="n">
+        <v>46.83</v>
+      </c>
       <c r="AJ7" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1253,6 +1268,9 @@
       <c r="AB8" t="n">
         <v>716534.88316</v>
       </c>
+      <c r="AC8" t="n">
+        <v>46.18</v>
+      </c>
       <c r="AJ8" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1330,6 +1348,9 @@
       <c r="AB9" t="n">
         <v>829159.4432</v>
       </c>
+      <c r="AC9" t="n">
+        <v>46.04</v>
+      </c>
       <c r="AJ9" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1407,6 +1428,9 @@
       <c r="AB10" t="n">
         <v>1594423.90222</v>
       </c>
+      <c r="AC10" t="n">
+        <v>45.59</v>
+      </c>
       <c r="AJ10" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1484,6 +1508,9 @@
       <c r="AB11" t="n">
         <v>789972.90392</v>
       </c>
+      <c r="AC11" t="n">
+        <v>50.43</v>
+      </c>
       <c r="AJ11" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1561,6 +1588,9 @@
       <c r="AB12" t="n">
         <v>2581808.51912</v>
       </c>
+      <c r="AC12" t="n">
+        <v>51.93</v>
+      </c>
       <c r="AJ12" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1638,6 +1668,9 @@
       <c r="AB13" t="n">
         <v>981579.05883</v>
       </c>
+      <c r="AC13" t="n">
+        <v>55.15</v>
+      </c>
       <c r="AJ13" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1715,6 +1748,9 @@
       <c r="AB14" t="n">
         <v>762823.51981</v>
       </c>
+      <c r="AC14" t="n">
+        <v>54.83</v>
+      </c>
       <c r="AJ14" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1792,6 +1828,9 @@
       <c r="AB15" t="n">
         <v>4503531.19663</v>
       </c>
+      <c r="AC15" t="n">
+        <v>54.66</v>
+      </c>
       <c r="AJ15" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1872,6 +1911,9 @@
       <c r="AB16" t="n">
         <v>9717927.89711</v>
       </c>
+      <c r="AC16" t="n">
+        <v>52.01</v>
+      </c>
       <c r="AJ16" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -1952,6 +1994,9 @@
       <c r="AB17" t="n">
         <v>13620381.48736</v>
       </c>
+      <c r="AC17" t="n">
+        <v>54.43</v>
+      </c>
       <c r="AJ17" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -2032,6 +2077,9 @@
       <c r="AB18" t="n">
         <v>4483317.54093</v>
       </c>
+      <c r="AC18" t="n">
+        <v>50.22</v>
+      </c>
       <c r="AJ18" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -2115,6 +2163,9 @@
       <c r="AB19" t="n">
         <v>2979494.89578</v>
       </c>
+      <c r="AC19" t="n">
+        <v>51.27</v>
+      </c>
       <c r="AJ19" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -2198,6 +2249,9 @@
       <c r="AB20" t="n">
         <v>7559250.35841</v>
       </c>
+      <c r="AC20" t="n">
+        <v>49.56</v>
+      </c>
       <c r="AJ20" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -2281,6 +2335,9 @@
       <c r="AB21" t="n">
         <v>3816424.84366</v>
       </c>
+      <c r="AC21" t="n">
+        <v>51.91</v>
+      </c>
       <c r="AJ21" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -2364,6 +2421,9 @@
       <c r="AB22" t="n">
         <v>1667068.5947</v>
       </c>
+      <c r="AC22" t="n">
+        <v>49.85</v>
+      </c>
       <c r="AJ22" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -2447,6 +2507,9 @@
       <c r="AB23" t="n">
         <v>2615428.9535</v>
       </c>
+      <c r="AC23" t="n">
+        <v>52.13</v>
+      </c>
       <c r="AJ23" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -2530,6 +2593,9 @@
       <c r="AB24" t="n">
         <v>1971541.38956</v>
       </c>
+      <c r="AC24" t="n">
+        <v>45.99</v>
+      </c>
       <c r="AJ24" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -2612,6 +2678,9 @@
       </c>
       <c r="AB25" t="n">
         <v>2362962.39597</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>45.47</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
@@ -2690,7 +2759,9 @@
       <c r="AB26" s="3" t="n">
         <v>2037632.16795</v>
       </c>
-      <c r="AC26" s="3" t="n"/>
+      <c r="AC26" s="3" t="n">
+        <v>46.95</v>
+      </c>
       <c r="AD26" s="3" t="n"/>
       <c r="AE26" s="3" t="n"/>
       <c r="AF26" s="3" t="n"/>
@@ -2779,7 +2850,9 @@
       <c r="AB27" s="3" t="n">
         <v>1103202.75839</v>
       </c>
-      <c r="AC27" s="3" t="n"/>
+      <c r="AC27" s="3" t="n">
+        <v>53.44</v>
+      </c>
       <c r="AD27" s="3" t="n"/>
       <c r="AE27" s="3" t="n"/>
       <c r="AF27" s="3" t="n"/>
@@ -2868,7 +2941,9 @@
       <c r="AB28" s="3" t="n">
         <v>2345884.3215</v>
       </c>
-      <c r="AC28" s="3" t="n"/>
+      <c r="AC28" s="3" t="n">
+        <v>50.02</v>
+      </c>
       <c r="AD28" s="3" t="n"/>
       <c r="AE28" s="3" t="n"/>
       <c r="AF28" s="3" t="n"/>
@@ -2963,6 +3038,9 @@
       <c r="AB29" t="n">
         <v>1483028.91662</v>
       </c>
+      <c r="AC29" t="n">
+        <v>49.14</v>
+      </c>
       <c r="AJ29" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3046,6 +3124,9 @@
       <c r="AB30" t="n">
         <v>1323596.82829</v>
       </c>
+      <c r="AC30" t="n">
+        <v>54.16</v>
+      </c>
       <c r="AJ30" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3129,6 +3210,9 @@
       <c r="AB31" t="n">
         <v>1541065.83729</v>
       </c>
+      <c r="AC31" t="n">
+        <v>43.04</v>
+      </c>
       <c r="AJ31" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3212,6 +3296,9 @@
       <c r="AB32" t="n">
         <v>2118286.95634</v>
       </c>
+      <c r="AC32" t="n">
+        <v>46.2</v>
+      </c>
       <c r="AJ32" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3295,6 +3382,9 @@
       <c r="AB33" t="n">
         <v>1013687.05613</v>
       </c>
+      <c r="AC33" t="n">
+        <v>42.61</v>
+      </c>
       <c r="AJ33" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3378,6 +3468,9 @@
       <c r="AB34" t="n">
         <v>535087.36674</v>
       </c>
+      <c r="AC34" t="n">
+        <v>47.45</v>
+      </c>
       <c r="AJ34" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3461,6 +3554,9 @@
       <c r="AB35" t="n">
         <v>1688089.23149</v>
       </c>
+      <c r="AC35" t="n">
+        <v>46.54</v>
+      </c>
       <c r="AJ35" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3544,6 +3640,9 @@
       <c r="AB36" t="n">
         <v>860103.143</v>
       </c>
+      <c r="AC36" t="n">
+        <v>48.23</v>
+      </c>
       <c r="AJ36" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3627,6 +3726,9 @@
       <c r="AB37" t="n">
         <v>957955.40446</v>
       </c>
+      <c r="AC37" t="n">
+        <v>44.68</v>
+      </c>
       <c r="AJ37" t="inlineStr">
         <is>
           <t>DELISTED</t>
@@ -3709,6 +3811,9 @@
       </c>
       <c r="AB38" t="n">
         <v>4776726.25304</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>50.65</v>
       </c>
       <c r="AJ38" t="inlineStr">
         <is>

</xml_diff>